<commit_message>
Pazy wing LCO analysis
</commit_message>
<xml_diff>
--- a/lib/WingPropellerUVLM/examples/pazy_aerobeams_coupled/output/stability_sweep/damping_estimation.xlsx
+++ b/lib/WingPropellerUVLM/examples/pazy_aerobeams_coupled/output/stability_sweep/damping_estimation.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Documents\João Tavares\Doutorado EESC\Models\AeroBeams_UVLM.jl\lib\WingPropellerUVLM\examples\pazy_aerobeams_coupled\output\stability_sweep\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103929B9-A6DA-4CFB-B464-DA4E921B3A78}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4B01CF-D3DC-4ABD-97F0-909B0FDCE5B6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{DC610DD0-7593-4B9B-A937-5F71CD1E14EB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{DC610DD0-7593-4B9B-A937-5F71CD1E14EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1421,11 +1420,12 @@
   <cols>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.28515625" customWidth="1"/>
-    <col min="10" max="11" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8.140625" customWidth="1"/>

</xml_diff>